<commit_message>
Update online max_rank calculation
</commit_message>
<xml_diff>
--- a/data/net_contest.xlsx
+++ b/data/net_contest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25420" windowHeight="16300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25600" windowHeight="10480" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="net1" sheetId="1" state="visible" r:id="rId1"/>
@@ -11,17 +11,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="net3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
-    <font>
-      <name val="宋体"/>
-      <family val="2"/>
+  <fonts count="23">
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -36,12 +36,164 @@
     <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <family val="3"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
+      <color theme="3"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF3F3F76"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FF3F3F3F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFA7D00"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF006100"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C0006"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF9C6500"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="0"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="34">
     <fill>
       <patternFill/>
     </fill>
@@ -54,8 +206,194 @@
         <bgColor rgb="FF4472C4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -63,18 +401,311 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="49">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="千位分隔" xfId="1" builtinId="3"/>
+    <cellStyle name="货币" xfId="2" builtinId="4"/>
+    <cellStyle name="百分比" xfId="3" builtinId="5"/>
+    <cellStyle name="千位分隔[0]" xfId="4" builtinId="6"/>
+    <cellStyle name="货币[0]" xfId="5" builtinId="7"/>
+    <cellStyle name="超链接" xfId="6" builtinId="8"/>
+    <cellStyle name="已访问的超链接" xfId="7" builtinId="9"/>
+    <cellStyle name="注释" xfId="8" builtinId="10"/>
+    <cellStyle name="警告文本" xfId="9" builtinId="11"/>
+    <cellStyle name="标题" xfId="10" builtinId="15"/>
+    <cellStyle name="解释性文本" xfId="11" builtinId="53"/>
+    <cellStyle name="标题 1" xfId="12" builtinId="16"/>
+    <cellStyle name="标题 2" xfId="13" builtinId="17"/>
+    <cellStyle name="标题 3" xfId="14" builtinId="18"/>
+    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
+    <cellStyle name="输入" xfId="16" builtinId="20"/>
+    <cellStyle name="输出" xfId="17" builtinId="21"/>
+    <cellStyle name="计算" xfId="18" builtinId="22"/>
+    <cellStyle name="检查单元格" xfId="19" builtinId="23"/>
+    <cellStyle name="链接单元格" xfId="20" builtinId="24"/>
+    <cellStyle name="汇总" xfId="21" builtinId="25"/>
+    <cellStyle name="好" xfId="22" builtinId="26"/>
+    <cellStyle name="差" xfId="23" builtinId="27"/>
+    <cellStyle name="适中" xfId="24" builtinId="28"/>
+    <cellStyle name="强调文字颜色 1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - 强调文字颜色 1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - 强调文字颜色 1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - 强调文字颜色 1" xfId="28" builtinId="32"/>
+    <cellStyle name="强调文字颜色 2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - 强调文字颜色 2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - 强调文字颜色 2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - 强调文字颜色 2" xfId="32" builtinId="36"/>
+    <cellStyle name="强调文字颜色 3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - 强调文字颜色 3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - 强调文字颜色 3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - 强调文字颜色 3" xfId="36" builtinId="40"/>
+    <cellStyle name="强调文字颜色 4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - 强调文字颜色 4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - 强调文字颜色 4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - 强调文字颜色 4" xfId="40" builtinId="44"/>
+    <cellStyle name="强调文字颜色 5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - 强调文字颜色 5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - 强调文字颜色 5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - 强调文字颜色 5" xfId="44" builtinId="48"/>
+    <cellStyle name="强调文字颜色 6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - 强调文字颜色 6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -427,7 +1058,6 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -437,8 +1067,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -475,6 +1105,11 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>max_rank</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>得分</t>
         </is>
       </c>
@@ -500,7 +1135,10 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>38.05</v>
+        <v>2486</v>
+      </c>
+      <c r="G2" t="n">
+        <v>45.19</v>
       </c>
     </row>
     <row r="3">
@@ -524,7 +1162,10 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>1.9</v>
+        <v>2486</v>
+      </c>
+      <c r="G3" t="n">
+        <v>20.69</v>
       </c>
     </row>
     <row r="4">
@@ -548,7 +1189,10 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>50.4</v>
+        <v>2486</v>
+      </c>
+      <c r="G4" t="n">
+        <v>55.14</v>
       </c>
     </row>
     <row r="5">
@@ -572,7 +1216,10 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>70.8</v>
+        <v>2486</v>
+      </c>
+      <c r="G5" t="n">
+        <v>73.31</v>
       </c>
     </row>
     <row r="6">
@@ -596,7 +1243,10 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>35.75</v>
+        <v>2486</v>
+      </c>
+      <c r="G6" t="n">
+        <v>44.27</v>
       </c>
     </row>
     <row r="7">
@@ -620,7 +1270,10 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>34.35</v>
+        <v>2486</v>
+      </c>
+      <c r="G7" t="n">
+        <v>43.7</v>
       </c>
     </row>
     <row r="8">
@@ -644,7 +1297,10 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>26.6</v>
+        <v>2486</v>
+      </c>
+      <c r="G8" t="n">
+        <v>40.59</v>
       </c>
     </row>
     <row r="9">
@@ -668,7 +1324,10 @@
         <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>61.53</v>
+        <v>2486</v>
+      </c>
+      <c r="G9" t="n">
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="10">
@@ -692,7 +1351,10 @@
         <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>36.7</v>
+        <v>2486</v>
+      </c>
+      <c r="G10" t="n">
+        <v>44.65</v>
       </c>
     </row>
     <row r="11">
@@ -716,7 +1378,10 @@
         <v>12</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>2486</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18.97</v>
       </c>
     </row>
     <row r="12">
@@ -740,7 +1405,10 @@
         <v>12</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2486</v>
+      </c>
+      <c r="G12" t="n">
+        <v>17.42</v>
       </c>
     </row>
     <row r="13">
@@ -764,7 +1432,10 @@
         <v>12</v>
       </c>
       <c r="F13" t="n">
-        <v>13.92</v>
+        <v>2486</v>
+      </c>
+      <c r="G13" t="n">
+        <v>30.5</v>
       </c>
     </row>
     <row r="14">
@@ -787,6 +1458,9 @@
         <v>12</v>
       </c>
       <c r="F14" t="n">
+        <v>2486</v>
+      </c>
+      <c r="G14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -802,7 +1476,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
@@ -1011,7 +1685,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>

</xml_diff>